<commit_message>
fix(m044): unblock manuscript patching for Discussion + Limitations
- Match opening Discussion paragraph through 'Three findings' anchor; keep
  fallbacks for legacy phrasing.
- Drive Cox wording from gross-vs-microscopic HR/p (elevated hazard vs NS).
- Replace era-span sentence with mig_258 strata counts plus supplement clause;
  narrow surgery-date % replacement for Limitations only.
- Guard calendar-strata logic on column presence; collapse extra blank lines
  after Discussion opener.
- Remove stray f-prefix strings; submission package script copy updated.
- Refresh workbook, inclusion flow QC CSV, manuscript, and selected figures.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/M044_ETE_tables.xlsx
+++ b/M044_ETE_tables.xlsx
@@ -8679,7 +8679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:E214"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="70" customWidth="1" style="18" min="1" max="1"/>
@@ -9274,97 +9274,1921 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="18" t="inlineStr">
         <is>
           <t>S4 pooled-LVI artifact check</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="18" t="inlineStr">
         <is>
           <t>OR pooled=1.7360199189525616 p=0.0010321630526339087</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="18" t="inlineStr">
         <is>
           <t>protective_sig=False; pooled_OR&gt;1_sig=True</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '1.1-2'): got 6.29% expected 4.1% (n=318)</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '2.1-4'): got 12.5% expected 7.0% (n=344)</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&lt;=1'): got 4.48% expected 2.6% (n=268)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&gt;4'): got 12.2% expected 8.6% (n=336)</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '1.1-2'): got 3.65% expected 2.7% (n=712)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '2.1-4'): got 3.58% expected 2.3% (n=642)</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&lt;=1'): got 2.01% expected 1.1% (n=947)</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&gt;4'): got 7.06% expected 5.6% (n=269)</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '1.1-2'): got 22.73% expected 11.4% (n=44)</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '2.1-4'): got 11.63% expected 7.0% (n=43)</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '&gt;4'): got 13.21% expected 3.8% (n=53)</t>
         </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="18" t="inlineStr">
+        <is>
+          <t>S4 pooled-LVI artifact check</t>
+        </is>
+      </c>
+      <c r="B60" s="18" t="inlineStr">
+        <is>
+          <t>OR pooled=1.7360199189525616 p=0.0010321630526339087</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>protective_sig=False; pooled_OR&gt;1_sig=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '1.1-2'): got 6.29% expected 4.1% (n=318)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '2.1-4'): got 12.5% expected 7.0% (n=344)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&lt;=1'): got 4.48% expected 2.6% (n=268)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&gt;4'): got 12.2% expected 8.6% (n=336)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '1.1-2'): got 3.65% expected 2.7% (n=712)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '2.1-4'): got 3.58% expected 2.3% (n=642)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&lt;=1'): got 2.01% expected 1.1% (n=947)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&gt;4'): got 7.06% expected 5.6% (n=269)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '1.1-2'): got 22.73% expected 11.4% (n=44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '2.1-4'): got 11.63% expected 7.0% (n=43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '&gt;4'): got 13.21% expected 3.8% (n=53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="31" t="inlineStr">
+        <is>
+          <t>Strict-DTC Cox/KM inclusion flow</t>
+        </is>
+      </c>
+      <c r="B74" s="18" t="inlineStr">
+        <is>
+          <t>/Users/ros/THyroid 2026/data/m044/m044_inclusion_flow_qc.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="B75" s="18" t="inlineStr">
+        <is>
+          <t>criterion</t>
+        </is>
+      </c>
+      <c r="C75" s="18" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>excluded_at_step</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="inlineStr">
+        <is>
+          <t>cum_excluded_from_cohort</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t>M044 analytic extract (cohort_m044_ajcc_ete_v1 + recurrence join)</t>
+        </is>
+      </c>
+      <c r="C76" s="18" t="n">
+        <v>4128</v>
+      </c>
+      <c r="D76" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t>Strict-DTC (exclude MTC/anaplastic/NIFTP/FTUMP/benign-neoplasm list per script)</t>
+        </is>
+      </c>
+      <c r="C77" s="18" t="n">
+        <v>3789</v>
+      </c>
+      <c r="D77" s="18" t="n">
+        <v>339</v>
+      </c>
+      <c r="E77" s="18" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B78" s="18" t="inlineStr">
+        <is>
+          <t>Three-level ETE (No/negative vs Microscopic vs Gross)</t>
+        </is>
+      </c>
+      <c r="C78" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D78" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="E78" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t>Sex known (female/male — multivariable frame)</t>
+        </is>
+      </c>
+      <c r="C79" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D79" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B80" s="18" t="inlineStr">
+        <is>
+          <t>Positive follow-up (followup_years &gt; 0)</t>
+        </is>
+      </c>
+      <c r="C80" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D80" s="18" t="n">
+        <v>1231</v>
+      </c>
+      <c r="E80" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B81" s="18" t="inlineStr">
+        <is>
+          <t>Known surgery date (surg_first_date non-null — CPM SSOT lineage)</t>
+        </is>
+      </c>
+      <c r="C81" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D81" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B82" s="18" t="inlineStr">
+        <is>
+          <t>Finite positive Cox duration (days; event-time or censored PY)</t>
+        </is>
+      </c>
+      <c r="C82" s="18" t="n">
+        <v>2494</v>
+      </c>
+      <c r="D82" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="E82" s="18" t="n">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B83" s="18" t="inlineStr">
+        <is>
+          <t>Age + tumor size non-missing (Cox covariate complete-case)</t>
+        </is>
+      </c>
+      <c r="C83" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D83" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E83" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B84" s="18" t="inlineStr">
+        <is>
+          <t>Final Cox PH / KM analytic rows (= step 7; lifelines fitted sample)</t>
+        </is>
+      </c>
+      <c r="C84" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D84" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="18" t="inlineStr">
+        <is>
+          <t>S4 pooled-LVI artifact check</t>
+        </is>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
+        <is>
+          <t>OR pooled=1.7360199189525616 p=0.0010321630526339087</t>
+        </is>
+      </c>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>protective_sig=False; pooled_OR&gt;1_sig=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '1.1-2'): got 6.29% expected 4.1% (n=318)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '2.1-4'): got 12.5% expected 7.0% (n=344)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&lt;=1'): got 4.48% expected 2.6% (n=268)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&gt;4'): got 12.2% expected 8.6% (n=336)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '1.1-2'): got 3.65% expected 2.7% (n=712)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '2.1-4'): got 3.58% expected 2.3% (n=642)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&lt;=1'): got 2.01% expected 1.1% (n=947)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&gt;4'): got 7.06% expected 5.6% (n=269)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '1.1-2'): got 22.73% expected 11.4% (n=44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '2.1-4'): got 11.63% expected 7.0% (n=43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '&gt;4'): got 13.21% expected 3.8% (n=53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="31" t="inlineStr">
+        <is>
+          <t>Strict-DTC Cox/KM inclusion flow</t>
+        </is>
+      </c>
+      <c r="B100" s="18" t="inlineStr">
+        <is>
+          <t>/Users/ros/THyroid 2026/data/m044/m044_inclusion_flow_qc.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="18" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="B101" s="18" t="inlineStr">
+        <is>
+          <t>criterion</t>
+        </is>
+      </c>
+      <c r="C101" s="18" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D101" s="18" t="inlineStr">
+        <is>
+          <t>excluded_at_step</t>
+        </is>
+      </c>
+      <c r="E101" s="18" t="inlineStr">
+        <is>
+          <t>cum_excluded_from_cohort</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="B102" s="18" t="inlineStr">
+        <is>
+          <t>M044 analytic extract (cohort_m044_ajcc_ete_v1 + recurrence join)</t>
+        </is>
+      </c>
+      <c r="C102" s="18" t="n">
+        <v>4128</v>
+      </c>
+      <c r="D102" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B103" s="18" t="inlineStr">
+        <is>
+          <t>Strict-DTC (exclude MTC/anaplastic/NIFTP/FTUMP/benign-neoplasm list per script)</t>
+        </is>
+      </c>
+      <c r="C103" s="18" t="n">
+        <v>3789</v>
+      </c>
+      <c r="D103" s="18" t="n">
+        <v>339</v>
+      </c>
+      <c r="E103" s="18" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B104" s="18" t="inlineStr">
+        <is>
+          <t>Three-level ETE (No/negative vs Microscopic vs Gross)</t>
+        </is>
+      </c>
+      <c r="C104" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D104" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="E104" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B105" s="18" t="inlineStr">
+        <is>
+          <t>Sex known (female/male — multivariable frame)</t>
+        </is>
+      </c>
+      <c r="C105" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D105" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B106" s="18" t="inlineStr">
+        <is>
+          <t>Positive follow-up (followup_years &gt; 0)</t>
+        </is>
+      </c>
+      <c r="C106" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D106" s="18" t="n">
+        <v>1231</v>
+      </c>
+      <c r="E106" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B107" s="18" t="inlineStr">
+        <is>
+          <t>Known surgery date (surg_first_date non-null — CPM SSOT lineage)</t>
+        </is>
+      </c>
+      <c r="C107" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D107" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B108" s="18" t="inlineStr">
+        <is>
+          <t>Finite positive Cox duration (days; event-time or censored PY)</t>
+        </is>
+      </c>
+      <c r="C108" s="18" t="n">
+        <v>2494</v>
+      </c>
+      <c r="D108" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="E108" s="18" t="n">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B109" s="18" t="inlineStr">
+        <is>
+          <t>Age + tumor size non-missing (Cox covariate complete-case)</t>
+        </is>
+      </c>
+      <c r="C109" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D109" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E109" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B110" s="18" t="inlineStr">
+        <is>
+          <t>Final Cox PH / KM analytic rows (= step 7; lifelines fitted sample)</t>
+        </is>
+      </c>
+      <c r="C110" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D110" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="18" t="inlineStr">
+        <is>
+          <t>S4 pooled-LVI artifact check</t>
+        </is>
+      </c>
+      <c r="B112" s="18" t="inlineStr">
+        <is>
+          <t>OR pooled=1.7360199189525616 p=0.0010321630526339087</t>
+        </is>
+      </c>
+      <c r="C112" s="18" t="inlineStr">
+        <is>
+          <t>protective_sig=False; pooled_OR&gt;1_sig=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '1.1-2'): got 6.29% expected 4.1% (n=318)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '2.1-4'): got 12.5% expected 7.0% (n=344)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&lt;=1'): got 4.48% expected 2.6% (n=268)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&gt;4'): got 12.2% expected 8.6% (n=336)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '1.1-2'): got 3.65% expected 2.7% (n=712)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '2.1-4'): got 3.58% expected 2.3% (n=642)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&lt;=1'): got 2.01% expected 1.1% (n=947)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&gt;4'): got 7.06% expected 5.6% (n=269)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '1.1-2'): got 22.73% expected 11.4% (n=44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '2.1-4'): got 11.63% expected 7.0% (n=43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '&gt;4'): got 13.21% expected 3.8% (n=53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="31" t="inlineStr">
+        <is>
+          <t>Strict-DTC Cox/KM inclusion flow</t>
+        </is>
+      </c>
+      <c r="B126" s="18" t="inlineStr">
+        <is>
+          <t>/Users/ros/THyroid 2026/data/m044/m044_inclusion_flow_qc.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="18" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="B127" s="18" t="inlineStr">
+        <is>
+          <t>criterion</t>
+        </is>
+      </c>
+      <c r="C127" s="18" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D127" s="18" t="inlineStr">
+        <is>
+          <t>excluded_at_step</t>
+        </is>
+      </c>
+      <c r="E127" s="18" t="inlineStr">
+        <is>
+          <t>cum_excluded_from_cohort</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="B128" s="18" t="inlineStr">
+        <is>
+          <t>M044 analytic extract (cohort_m044_ajcc_ete_v1 + recurrence join)</t>
+        </is>
+      </c>
+      <c r="C128" s="18" t="n">
+        <v>4128</v>
+      </c>
+      <c r="D128" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E128" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B129" s="18" t="inlineStr">
+        <is>
+          <t>Strict-DTC (exclude MTC/anaplastic/NIFTP/FTUMP/benign-neoplasm list per script)</t>
+        </is>
+      </c>
+      <c r="C129" s="18" t="n">
+        <v>3789</v>
+      </c>
+      <c r="D129" s="18" t="n">
+        <v>339</v>
+      </c>
+      <c r="E129" s="18" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B130" s="18" t="inlineStr">
+        <is>
+          <t>Three-level ETE (No/negative vs Microscopic vs Gross)</t>
+        </is>
+      </c>
+      <c r="C130" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D130" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="E130" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B131" s="18" t="inlineStr">
+        <is>
+          <t>Sex known (female/male — multivariable frame)</t>
+        </is>
+      </c>
+      <c r="C131" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D131" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B132" s="18" t="inlineStr">
+        <is>
+          <t>Positive follow-up (followup_years &gt; 0)</t>
+        </is>
+      </c>
+      <c r="C132" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D132" s="18" t="n">
+        <v>1231</v>
+      </c>
+      <c r="E132" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B133" s="18" t="inlineStr">
+        <is>
+          <t>Known surgery date (surg_first_date non-null — CPM SSOT lineage)</t>
+        </is>
+      </c>
+      <c r="C133" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D133" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B134" s="18" t="inlineStr">
+        <is>
+          <t>Finite positive Cox duration (days; event-time or censored PY)</t>
+        </is>
+      </c>
+      <c r="C134" s="18" t="n">
+        <v>2494</v>
+      </c>
+      <c r="D134" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="E134" s="18" t="n">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B135" s="18" t="inlineStr">
+        <is>
+          <t>Age + tumor size non-missing (Cox covariate complete-case)</t>
+        </is>
+      </c>
+      <c r="C135" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D135" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E135" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B136" s="18" t="inlineStr">
+        <is>
+          <t>Final Cox PH / KM analytic rows (= step 7; lifelines fitted sample)</t>
+        </is>
+      </c>
+      <c r="C136" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D136" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E136" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="18" t="inlineStr">
+        <is>
+          <t>S4 pooled-LVI artifact check</t>
+        </is>
+      </c>
+      <c r="B138" s="18" t="inlineStr">
+        <is>
+          <t>OR pooled=1.7360199189525616 p=0.0010321630526339087</t>
+        </is>
+      </c>
+      <c r="C138" s="18" t="inlineStr">
+        <is>
+          <t>protective_sig=False; pooled_OR&gt;1_sig=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '1.1-2'): got 6.29% expected 4.1% (n=318)</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '2.1-4'): got 12.5% expected 7.0% (n=344)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&lt;=1'): got 4.48% expected 2.6% (n=268)</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&gt;4'): got 12.2% expected 8.6% (n=336)</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '1.1-2'): got 3.65% expected 2.7% (n=712)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '2.1-4'): got 3.58% expected 2.3% (n=642)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&lt;=1'): got 2.01% expected 1.1% (n=947)</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&gt;4'): got 7.06% expected 5.6% (n=269)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '1.1-2'): got 22.73% expected 11.4% (n=44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '2.1-4'): got 11.63% expected 7.0% (n=43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '&gt;4'): got 13.21% expected 3.8% (n=53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="31" t="inlineStr">
+        <is>
+          <t>Strict-DTC Cox/KM inclusion flow</t>
+        </is>
+      </c>
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t>/Users/ros/THyroid 2026/data/m044/m044_inclusion_flow_qc.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="18" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="B153" s="18" t="inlineStr">
+        <is>
+          <t>criterion</t>
+        </is>
+      </c>
+      <c r="C153" s="18" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D153" s="18" t="inlineStr">
+        <is>
+          <t>excluded_at_step</t>
+        </is>
+      </c>
+      <c r="E153" s="18" t="inlineStr">
+        <is>
+          <t>cum_excluded_from_cohort</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="B154" s="18" t="inlineStr">
+        <is>
+          <t>M044 analytic extract (cohort_m044_ajcc_ete_v1 + recurrence join)</t>
+        </is>
+      </c>
+      <c r="C154" s="18" t="n">
+        <v>4128</v>
+      </c>
+      <c r="D154" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B155" s="18" t="inlineStr">
+        <is>
+          <t>Strict-DTC (exclude MTC/anaplastic/NIFTP/FTUMP/benign-neoplasm list per script)</t>
+        </is>
+      </c>
+      <c r="C155" s="18" t="n">
+        <v>3789</v>
+      </c>
+      <c r="D155" s="18" t="n">
+        <v>339</v>
+      </c>
+      <c r="E155" s="18" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B156" s="18" t="inlineStr">
+        <is>
+          <t>Three-level ETE (No/negative vs Microscopic vs Gross)</t>
+        </is>
+      </c>
+      <c r="C156" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D156" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="E156" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B157" s="18" t="inlineStr">
+        <is>
+          <t>Sex known (female/male — multivariable frame)</t>
+        </is>
+      </c>
+      <c r="C157" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D157" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B158" s="18" t="inlineStr">
+        <is>
+          <t>Positive follow-up (followup_years &gt; 0)</t>
+        </is>
+      </c>
+      <c r="C158" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D158" s="18" t="n">
+        <v>1231</v>
+      </c>
+      <c r="E158" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B159" s="18" t="inlineStr">
+        <is>
+          <t>Known surgery date (surg_first_date non-null — CPM SSOT lineage)</t>
+        </is>
+      </c>
+      <c r="C159" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D159" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B160" s="18" t="inlineStr">
+        <is>
+          <t>Finite positive Cox duration (days; event-time or censored PY)</t>
+        </is>
+      </c>
+      <c r="C160" s="18" t="n">
+        <v>2494</v>
+      </c>
+      <c r="D160" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="E160" s="18" t="n">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B161" s="18" t="inlineStr">
+        <is>
+          <t>Age + tumor size non-missing (Cox covariate complete-case)</t>
+        </is>
+      </c>
+      <c r="C161" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D161" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E161" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B162" s="18" t="inlineStr">
+        <is>
+          <t>Final Cox PH / KM analytic rows (= step 7; lifelines fitted sample)</t>
+        </is>
+      </c>
+      <c r="C162" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D162" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E162" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="18" t="inlineStr">
+        <is>
+          <t>S4 pooled-LVI artifact check</t>
+        </is>
+      </c>
+      <c r="B164" s="18" t="inlineStr">
+        <is>
+          <t>OR pooled=1.7360199189525616 p=0.0010321630526339087</t>
+        </is>
+      </c>
+      <c r="C164" s="18" t="inlineStr">
+        <is>
+          <t>protective_sig=False; pooled_OR&gt;1_sig=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '1.1-2'): got 6.29% expected 4.1% (n=318)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '2.1-4'): got 12.5% expected 7.0% (n=344)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&lt;=1'): got 4.48% expected 2.6% (n=268)</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&gt;4'): got 12.2% expected 8.6% (n=336)</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '1.1-2'): got 3.65% expected 2.7% (n=712)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '2.1-4'): got 3.58% expected 2.3% (n=642)</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&lt;=1'): got 2.01% expected 1.1% (n=947)</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&gt;4'): got 7.06% expected 5.6% (n=269)</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '1.1-2'): got 22.73% expected 11.4% (n=44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '2.1-4'): got 11.63% expected 7.0% (n=43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="18" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '&gt;4'): got 13.21% expected 3.8% (n=53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="31" t="inlineStr">
+        <is>
+          <t>Strict-DTC Cox/KM inclusion flow</t>
+        </is>
+      </c>
+      <c r="B178" s="18" t="inlineStr">
+        <is>
+          <t>/Users/ros/THyroid 2026/data/m044/m044_inclusion_flow_qc.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="18" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="B179" s="18" t="inlineStr">
+        <is>
+          <t>criterion</t>
+        </is>
+      </c>
+      <c r="C179" s="18" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D179" s="18" t="inlineStr">
+        <is>
+          <t>excluded_at_step</t>
+        </is>
+      </c>
+      <c r="E179" s="18" t="inlineStr">
+        <is>
+          <t>cum_excluded_from_cohort</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="B180" s="18" t="inlineStr">
+        <is>
+          <t>M044 analytic extract (cohort_m044_ajcc_ete_v1 + recurrence join)</t>
+        </is>
+      </c>
+      <c r="C180" s="18" t="n">
+        <v>4128</v>
+      </c>
+      <c r="D180" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E180" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B181" s="18" t="inlineStr">
+        <is>
+          <t>Strict-DTC (exclude MTC/anaplastic/NIFTP/FTUMP/benign-neoplasm list per script)</t>
+        </is>
+      </c>
+      <c r="C181" s="18" t="n">
+        <v>3789</v>
+      </c>
+      <c r="D181" s="18" t="n">
+        <v>339</v>
+      </c>
+      <c r="E181" s="18" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B182" s="18" t="inlineStr">
+        <is>
+          <t>Three-level ETE (No/negative vs Microscopic vs Gross)</t>
+        </is>
+      </c>
+      <c r="C182" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D182" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="E182" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B183" s="18" t="inlineStr">
+        <is>
+          <t>Sex known (female/male — multivariable frame)</t>
+        </is>
+      </c>
+      <c r="C183" s="18" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D183" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E183" s="18" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B184" s="18" t="inlineStr">
+        <is>
+          <t>Positive follow-up (followup_years &gt; 0)</t>
+        </is>
+      </c>
+      <c r="C184" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D184" s="18" t="n">
+        <v>1231</v>
+      </c>
+      <c r="E184" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B185" s="18" t="inlineStr">
+        <is>
+          <t>Known surgery date (surg_first_date non-null — CPM SSOT lineage)</t>
+        </is>
+      </c>
+      <c r="C185" s="18" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D185" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E185" s="18" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B186" s="18" t="inlineStr">
+        <is>
+          <t>Finite positive Cox duration (days; event-time or censored PY)</t>
+        </is>
+      </c>
+      <c r="C186" s="18" t="n">
+        <v>2494</v>
+      </c>
+      <c r="D186" s="18" t="n">
+        <v>31</v>
+      </c>
+      <c r="E186" s="18" t="n">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B187" s="18" t="inlineStr">
+        <is>
+          <t>Age + tumor size non-missing (Cox covariate complete-case)</t>
+        </is>
+      </c>
+      <c r="C187" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D187" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E187" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B188" s="18" t="inlineStr">
+        <is>
+          <t>Final Cox PH / KM analytic rows (= step 7; lifelines fitted sample)</t>
+        </is>
+      </c>
+      <c r="C188" s="18" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D188" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E188" s="18" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>S4 pooled-LVI artifact check</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>OR pooled=1.7360199189525616 p=0.0010321630526339087</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>protective_sig=False; pooled_OR&gt;1_sig=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '1.1-2'): got 6.29% expected 4.1% (n=318)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '2.1-4'): got 12.5% expected 7.0% (n=344)</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&lt;=1'): got 4.48% expected 2.6% (n=268)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&gt;4'): got 12.2% expected 8.6% (n=336)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '1.1-2'): got 3.65% expected 2.7% (n=712)</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '2.1-4'): got 3.58% expected 2.3% (n=642)</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&lt;=1'): got 2.01% expected 1.1% (n=947)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&gt;4'): got 7.06% expected 5.6% (n=269)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '1.1-2'): got 22.73% expected 11.4% (n=44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '2.1-4'): got 11.63% expected 7.0% (n=43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '&gt;4'): got 13.21% expected 3.8% (n=53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="31" t="inlineStr">
+        <is>
+          <t>Strict-DTC Cox/KM inclusion flow</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>/Users/ros/THyroid 2026/data/m044/m044_inclusion_flow_qc.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>criterion</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>excluded_at_step</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>cum_excluded_from_cohort</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>0</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>M044 analytic extract (cohort_m044_ajcc_ete_v1 + recurrence join)</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>4128</v>
+      </c>
+      <c r="D206" t="n">
+        <v>0</v>
+      </c>
+      <c r="E206" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>1</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Strict-DTC (exclude MTC/anaplastic/NIFTP/FTUMP/benign-neoplasm list per script)</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>3789</v>
+      </c>
+      <c r="D207" t="n">
+        <v>339</v>
+      </c>
+      <c r="E207" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>2</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Three-level ETE (No/negative vs Microscopic vs Gross)</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D208" t="n">
+        <v>33</v>
+      </c>
+      <c r="E208" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>3</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Sex known (female/male — multivariable frame)</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D209" t="n">
+        <v>0</v>
+      </c>
+      <c r="E209" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>4</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Positive follow-up (followup_years &gt; 0)</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D210" t="n">
+        <v>1231</v>
+      </c>
+      <c r="E210" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>5</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Known surgery date (surg_first_date non-null — CPM SSOT lineage)</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D211" t="n">
+        <v>0</v>
+      </c>
+      <c r="E211" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>6</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Finite positive Cox duration (days; event-time or censored PY)</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>2494</v>
+      </c>
+      <c r="D212" t="n">
+        <v>31</v>
+      </c>
+      <c r="E212" t="n">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>7</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Age + tumor size non-missing (Cox covariate complete-case)</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D213" t="n">
+        <v>4</v>
+      </c>
+      <c r="E213" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>8</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Final Cox PH / KM analytic rows (= step 7; lifelines fitted sample)</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D214" t="n">
+        <v>0</v>
+      </c>
+      <c r="E214" t="n">
+        <v>1638</v>
       </c>
     </row>
   </sheetData>
@@ -12036,7 +13860,7 @@
       </c>
       <c r="J4" s="26" t="inlineStr">
         <is>
-          <t>Person-years</t>
+          <t>Person-years (FU&gt;0)</t>
         </is>
       </c>
       <c r="K4" s="26" t="inlineStr">
@@ -12070,27 +13894,27 @@
         <v>2576</v>
       </c>
       <c r="C5" s="28" t="n">
-        <v>59</v>
+        <v>87</v>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
-          <t>2.29%</t>
+          <t>3.38%</t>
         </is>
       </c>
       <c r="E5" s="28" t="n">
-        <v>86</v>
+        <v>13</v>
       </c>
       <c r="F5" s="28" t="inlineStr">
         <is>
-          <t>3.34%</t>
+          <t>0.50%</t>
         </is>
       </c>
       <c r="G5" s="28" t="n">
-        <v>145</v>
+        <v>100</v>
       </c>
       <c r="H5" s="28" t="inlineStr">
         <is>
-          <t>5.63%</t>
+          <t>3.88%</t>
         </is>
       </c>
       <c r="I5" s="28" t="n">
@@ -12100,7 +13924,7 @@
         <v>8137.3</v>
       </c>
       <c r="K5" s="28" t="n">
-        <v>0.73</v>
+        <v>1.03</v>
       </c>
       <c r="L5" s="28" t="n">
         <v>1.78</v>
@@ -12124,27 +13948,27 @@
         <v>1266</v>
       </c>
       <c r="C6" s="28" t="n">
-        <v>73</v>
+        <v>116</v>
       </c>
       <c r="D6" s="28" t="inlineStr">
         <is>
-          <t>5.77%</t>
+          <t>9.16%</t>
         </is>
       </c>
       <c r="E6" s="28" t="n">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="F6" s="28" t="inlineStr">
         <is>
-          <t>7.11%</t>
+          <t>0.63%</t>
         </is>
       </c>
       <c r="G6" s="28" t="n">
-        <v>163</v>
+        <v>124</v>
       </c>
       <c r="H6" s="28" t="inlineStr">
         <is>
-          <t>12.88%</t>
+          <t>9.79%</t>
         </is>
       </c>
       <c r="I6" s="28" t="n">
@@ -12154,7 +13978,7 @@
         <v>4138.3</v>
       </c>
       <c r="K6" s="28" t="n">
-        <v>1.76</v>
+        <v>2.73</v>
       </c>
       <c r="L6" s="28" t="n">
         <v>3.94</v>
@@ -12178,27 +14002,27 @@
         <v>192</v>
       </c>
       <c r="C7" s="28" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D7" s="28" t="inlineStr">
         <is>
-          <t>6.25%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="E7" s="28" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="F7" s="28" t="inlineStr">
         <is>
-          <t>8.85%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="G7" s="28" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="H7" s="28" t="inlineStr">
         <is>
-          <t>15.10%</t>
+          <t>13.02%</t>
         </is>
       </c>
       <c r="I7" s="28" t="n">
@@ -12208,7 +14032,7 @@
         <v>700.8</v>
       </c>
       <c r="K7" s="28" t="n">
-        <v>1.71</v>
+        <v>3.28</v>
       </c>
       <c r="L7" s="28" t="n">
         <v>4.14</v>
@@ -12333,7 +14157,7 @@
     <row r="11" ht="15" customHeight="1" s="19">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>Notes: Person-years use all follow-up time (incl zero-FU). Restricted to FU&gt;0 in Supp Table S3.</t>
+          <t>Notes: Col J sums follow-up years among patients with FU&gt;0 only (PY-rate denominator). Col K = 100 × (path-proven events among FU&gt;0) / col J. Path-proven n and Path-proven % include all patients (zero-FU retained in denominator for proportions).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M044: expand Cox/KM inclusion QC table and regenerate outputs
- Waterfall QC: strict-DTC, 3-level ETE, sex, FU>0, surgery date, Cox
  duration, tumor size, age; footer row with Cox n and path-proven events.
- Validate waterfall n matches build_cox_analytic_frame; add path_proven_events
  column and Excel QA column path_proven_events_final_only.
- Regenerate parquet, Cox summaries, workbook, patched manuscript Results,
  figures (via m044_make_figures).
- Supplement S3.2: drop stale 3212/914 denominators; point to mig_258 flags
  and validation runner.
- Submission package: sync script, Cox CSVs under 08_analysis_outputs, forest PNGs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/M044_ETE_tables.xlsx
+++ b/M044_ETE_tables.xlsx
@@ -8679,7 +8679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E214"/>
+  <dimension ref="A1:F241"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="70" customWidth="1" style="18" min="1" max="1"/>
@@ -10888,94 +10888,94 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" t="inlineStr">
+      <c r="A190" s="18" t="inlineStr">
         <is>
           <t>S4 pooled-LVI artifact check</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr">
+      <c r="B190" s="18" t="inlineStr">
         <is>
           <t>OR pooled=1.7360199189525616 p=0.0010321630526339087</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
+      <c r="C190" s="18" t="inlineStr">
         <is>
           <t>protective_sig=False; pooled_OR&gt;1_sig=True</t>
         </is>
       </c>
     </row>
     <row r="191">
-      <c r="A191" t="inlineStr">
+      <c r="A191" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '1.1-2'): got 6.29% expected 4.1% (n=318)</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="A192" t="inlineStr">
+      <c r="A192" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '2.1-4'): got 12.5% expected 7.0% (n=344)</t>
         </is>
       </c>
     </row>
     <row r="193">
-      <c r="A193" t="inlineStr">
+      <c r="A193" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&lt;=1'): got 4.48% expected 2.6% (n=268)</t>
         </is>
       </c>
     </row>
     <row r="194">
-      <c r="A194" t="inlineStr">
+      <c r="A194" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&gt;4'): got 12.2% expected 8.6% (n=336)</t>
         </is>
       </c>
     </row>
     <row r="195">
-      <c r="A195" t="inlineStr">
+      <c r="A195" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '1.1-2'): got 3.65% expected 2.7% (n=712)</t>
         </is>
       </c>
     </row>
     <row r="196">
-      <c r="A196" t="inlineStr">
+      <c r="A196" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '2.1-4'): got 3.58% expected 2.3% (n=642)</t>
         </is>
       </c>
     </row>
     <row r="197">
-      <c r="A197" t="inlineStr">
+      <c r="A197" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&lt;=1'): got 2.01% expected 1.1% (n=947)</t>
         </is>
       </c>
     </row>
     <row r="198">
-      <c r="A198" t="inlineStr">
+      <c r="A198" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&gt;4'): got 7.06% expected 5.6% (n=269)</t>
         </is>
       </c>
     </row>
     <row r="199">
-      <c r="A199" t="inlineStr">
+      <c r="A199" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '1.1-2'): got 22.73% expected 11.4% (n=44)</t>
         </is>
       </c>
     </row>
     <row r="200">
-      <c r="A200" t="inlineStr">
+      <c r="A200" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '2.1-4'): got 11.63% expected 7.0% (n=43)</t>
         </is>
       </c>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr">
+      <c r="A201" s="18" t="inlineStr">
         <is>
           <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '&gt;4'): got 13.21% expected 3.8% (n=53)</t>
         </is>
@@ -10987,208 +10987,539 @@
           <t>Strict-DTC Cox/KM inclusion flow</t>
         </is>
       </c>
-      <c r="B204" t="inlineStr">
+      <c r="B204" s="18" t="inlineStr">
         <is>
           <t>/Users/ros/THyroid 2026/data/m044/m044_inclusion_flow_qc.csv</t>
         </is>
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="inlineStr">
+      <c r="A205" s="18" t="inlineStr">
         <is>
           <t>step</t>
         </is>
       </c>
-      <c r="B205" t="inlineStr">
+      <c r="B205" s="18" t="inlineStr">
         <is>
           <t>criterion</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C205" s="18" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr">
+      <c r="D205" s="18" t="inlineStr">
         <is>
           <t>excluded_at_step</t>
         </is>
       </c>
-      <c r="E205" t="inlineStr">
+      <c r="E205" s="18" t="inlineStr">
         <is>
           <t>cum_excluded_from_cohort</t>
         </is>
       </c>
     </row>
     <row r="206">
-      <c r="A206" t="n">
+      <c r="A206" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="B206" t="inlineStr">
+      <c r="B206" s="18" t="inlineStr">
         <is>
           <t>M044 analytic extract (cohort_m044_ajcc_ete_v1 + recurrence join)</t>
         </is>
       </c>
-      <c r="C206" t="n">
+      <c r="C206" s="18" t="n">
         <v>4128</v>
       </c>
-      <c r="D206" t="n">
+      <c r="D206" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E206" t="n">
+      <c r="E206" s="18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="207">
-      <c r="A207" t="n">
+      <c r="A207" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B207" t="inlineStr">
+      <c r="B207" s="18" t="inlineStr">
         <is>
           <t>Strict-DTC (exclude MTC/anaplastic/NIFTP/FTUMP/benign-neoplasm list per script)</t>
         </is>
       </c>
-      <c r="C207" t="n">
+      <c r="C207" s="18" t="n">
         <v>3789</v>
       </c>
-      <c r="D207" t="n">
+      <c r="D207" s="18" t="n">
         <v>339</v>
       </c>
-      <c r="E207" t="n">
+      <c r="E207" s="18" t="n">
         <v>339</v>
       </c>
     </row>
     <row r="208">
-      <c r="A208" t="n">
+      <c r="A208" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B208" t="inlineStr">
+      <c r="B208" s="18" t="inlineStr">
         <is>
           <t>Three-level ETE (No/negative vs Microscopic vs Gross)</t>
         </is>
       </c>
-      <c r="C208" t="n">
+      <c r="C208" s="18" t="n">
         <v>3756</v>
       </c>
-      <c r="D208" t="n">
+      <c r="D208" s="18" t="n">
         <v>33</v>
       </c>
-      <c r="E208" t="n">
+      <c r="E208" s="18" t="n">
         <v>372</v>
       </c>
     </row>
     <row r="209">
-      <c r="A209" t="n">
+      <c r="A209" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B209" t="inlineStr">
+      <c r="B209" s="18" t="inlineStr">
         <is>
           <t>Sex known (female/male — multivariable frame)</t>
         </is>
       </c>
-      <c r="C209" t="n">
+      <c r="C209" s="18" t="n">
         <v>3756</v>
       </c>
-      <c r="D209" t="n">
+      <c r="D209" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E209" t="n">
+      <c r="E209" s="18" t="n">
         <v>372</v>
       </c>
     </row>
     <row r="210">
-      <c r="A210" t="n">
+      <c r="A210" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B210" t="inlineStr">
+      <c r="B210" s="18" t="inlineStr">
         <is>
           <t>Positive follow-up (followup_years &gt; 0)</t>
         </is>
       </c>
-      <c r="C210" t="n">
+      <c r="C210" s="18" t="n">
         <v>2525</v>
       </c>
-      <c r="D210" t="n">
+      <c r="D210" s="18" t="n">
         <v>1231</v>
       </c>
-      <c r="E210" t="n">
+      <c r="E210" s="18" t="n">
         <v>1603</v>
       </c>
     </row>
     <row r="211">
-      <c r="A211" t="n">
+      <c r="A211" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B211" t="inlineStr">
+      <c r="B211" s="18" t="inlineStr">
         <is>
           <t>Known surgery date (surg_first_date non-null — CPM SSOT lineage)</t>
         </is>
       </c>
-      <c r="C211" t="n">
+      <c r="C211" s="18" t="n">
         <v>2525</v>
       </c>
-      <c r="D211" t="n">
+      <c r="D211" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E211" t="n">
+      <c r="E211" s="18" t="n">
         <v>1603</v>
       </c>
     </row>
     <row r="212">
-      <c r="A212" t="n">
+      <c r="A212" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B212" t="inlineStr">
+      <c r="B212" s="18" t="inlineStr">
         <is>
           <t>Finite positive Cox duration (days; event-time or censored PY)</t>
         </is>
       </c>
-      <c r="C212" t="n">
+      <c r="C212" s="18" t="n">
         <v>2494</v>
       </c>
-      <c r="D212" t="n">
+      <c r="D212" s="18" t="n">
         <v>31</v>
       </c>
-      <c r="E212" t="n">
+      <c r="E212" s="18" t="n">
         <v>1634</v>
       </c>
     </row>
     <row r="213">
-      <c r="A213" t="n">
+      <c r="A213" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="B213" t="inlineStr">
+      <c r="B213" s="18" t="inlineStr">
         <is>
           <t>Age + tumor size non-missing (Cox covariate complete-case)</t>
         </is>
       </c>
-      <c r="C213" t="n">
+      <c r="C213" s="18" t="n">
         <v>2490</v>
       </c>
-      <c r="D213" t="n">
+      <c r="D213" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="E213" t="n">
+      <c r="E213" s="18" t="n">
         <v>1638</v>
       </c>
     </row>
     <row r="214">
-      <c r="A214" t="n">
+      <c r="A214" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="B214" t="inlineStr">
+      <c r="B214" s="18" t="inlineStr">
         <is>
           <t>Final Cox PH / KM analytic rows (= step 7; lifelines fitted sample)</t>
         </is>
       </c>
-      <c r="C214" t="n">
+      <c r="C214" s="18" t="n">
         <v>2490</v>
       </c>
-      <c r="D214" t="n">
+      <c r="D214" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E214" t="n">
+      <c r="E214" s="18" t="n">
         <v>1638</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>S4 pooled-LVI artifact check</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>OR pooled=1.7360199189525616 p=0.0010321630526339087</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>protective_sig=False; pooled_OR&gt;1_sig=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '1.1-2'): got 6.29% expected 4.1% (n=318)</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '2.1-4'): got 12.5% expected 7.0% (n=344)</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&lt;=1'): got 4.48% expected 2.6% (n=268)</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Gross ETE', '&gt;4'): got 12.2% expected 8.6% (n=336)</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '1.1-2'): got 3.65% expected 2.7% (n=712)</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '2.1-4'): got 3.58% expected 2.3% (n=642)</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&lt;=1'): got 2.01% expected 1.1% (n=947)</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('Microscopic ETE', '&gt;4'): got 7.06% expected 5.6% (n=269)</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '1.1-2'): got 22.73% expected 11.4% (n=44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '2.1-4'): got 11.63% expected 7.0% (n=43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>SIZE_STRAT_MISMATCH: ('No/negative ETE', '&gt;4'): got 13.21% expected 3.8% (n=53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="31" t="inlineStr">
+        <is>
+          <t>Strict-DTC Cox/KM inclusion flow</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>/Users/ros/THyroid 2026/data/m044/m044_inclusion_flow_qc.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>criterion</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>excluded_at_step</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>cum_excluded_from_cohort</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>path_proven_events_final_only</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>0</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>M044 analytic extract (cohort_m044_ajcc_ete_v1 + recurrence join)</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>4128</v>
+      </c>
+      <c r="D232" t="n">
+        <v>0</v>
+      </c>
+      <c r="E232" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>1</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Strict-DTC histology (exclude MTC/anaplastic/NIFTP/FTUMP/benign-neoplasm list)</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>3789</v>
+      </c>
+      <c r="D233" t="n">
+        <v>339</v>
+      </c>
+      <c r="E233" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>2</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Three-level ETE (No/negative vs Microscopic vs Gross)</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D234" t="n">
+        <v>33</v>
+      </c>
+      <c r="E234" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>3</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Sex known female/male (same frame as primary logistic/Cox categoricals)</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>3756</v>
+      </c>
+      <c r="D235" t="n">
+        <v>0</v>
+      </c>
+      <c r="E235" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>4</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Positive analytic follow-up (followup_years &gt; 0)</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D236" t="n">
+        <v>1231</v>
+      </c>
+      <c r="E236" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>5</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Known surgery date (CPM surg_first_date; mig_258/mig_254 lineage)</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>2525</v>
+      </c>
+      <c r="D237" t="n">
+        <v>0</v>
+      </c>
+      <c r="E237" t="n">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>6</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Finite positive Cox time_days (path-proven TTE if event else censor at FU×365.25)</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>2494</v>
+      </c>
+      <c r="D238" t="n">
+        <v>31</v>
+      </c>
+      <c r="E238" t="n">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>7</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Tumor size known (cm; Cox covariate complete-case)</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D239" t="n">
+        <v>4</v>
+      </c>
+      <c r="E239" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>8</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Age at surgery known (Cox covariate complete-case)</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D240" t="n">
+        <v>0</v>
+      </c>
+      <c r="E240" t="n">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>9</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Final Cox PH + Kaplan–Meier rows (lifelines sample; aligns Figure 6)</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>2490</v>
+      </c>
+      <c r="D241" t="n">
+        <v>0</v>
+      </c>
+      <c r="E241" t="n">
+        <v>1638</v>
+      </c>
+      <c r="F241" t="n">
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -13918,7 +14249,7 @@
         </is>
       </c>
       <c r="I5" s="28" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J5" s="28" t="n">
         <v>8137.3</v>
@@ -13972,7 +14303,7 @@
         </is>
       </c>
       <c r="I6" s="28" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="J6" s="28" t="n">
         <v>4138.3</v>
@@ -14026,7 +14357,7 @@
         </is>
       </c>
       <c r="I7" s="28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J7" s="28" t="n">
         <v>700.8</v>

</xml_diff>